<commit_message>
add session excel import/export template
</commit_message>
<xml_diff>
--- a/SourceCode/face-attendance-system/backend/templates/attendance-template.xlsx
+++ b/SourceCode/face-attendance-system/backend/templates/attendance-template.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Hocphan_PTIT\Bài tập lớn\TTCS\SourceCode\face-attendance-system\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698B34C8-9802-4F52-BE58-778A837AEAC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3BB5AA9-E738-4152-AB75-9457B6627D61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Kết quả điểm danh" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -131,11 +131,11 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -428,18 +428,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
     </row>
     <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>

</xml_diff>